<commit_message>
Update organization name, logo, and dropdown styles on member registration form
Replaces "الجمعية القلبية السورية" with "الرابطة السورية لأمراض وجراحة القلب", updates the logo from an emoji to a JPG image, and adjusts CSS for dropdowns to ensure visibility in dark and light modes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: fb83f075-83bf-4666-98f0-ea4bec10fd72
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f3968623-1a81-41d6-8213-67e89b7fa20e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/3a6f4480-5f60-41f1-9683-8e05aff8235c/fb83f075-83bf-4666-98f0-ea4bec10fd72/kJIIsq2
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/نموذج-الأعضاء-عربي.xlsx
+++ b/docs/form_by_n8n/نموذج-الأعضاء-عربي.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,159 @@
         <v>تاريخ التسجيل</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ابراهيم</v>
+      </c>
+      <c r="B2" t="str">
+        <v>الصيداوي</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D2" t="str">
+        <v>محمد علي</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G2" t="str">
+        <v>ذكر</v>
+      </c>
+      <c r="H2" t="str">
+        <v>جراحة قلب</v>
+      </c>
+      <c r="I2" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K2" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="L2" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="N2" t="str">
+        <v>عضو أصيل</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-05-05T17:26:35.077Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ابراهيم</v>
+      </c>
+      <c r="B3" t="str">
+        <v>الصيداوي</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D3" t="str">
+        <v>محمد علي</v>
+      </c>
+      <c r="E3" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F3" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G3" t="str">
+        <v>ذكر</v>
+      </c>
+      <c r="H3" t="str">
+        <v>جراحة قلب</v>
+      </c>
+      <c r="I3" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J3" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K3" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="L3" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="N3" t="str">
+        <v>عضو أصيل</v>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v>2026-05-05T17:35:01.976Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ابراهيم</v>
+      </c>
+      <c r="B4" t="str">
+        <v>الصيداوي</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D4" t="str">
+        <v>محمد علي</v>
+      </c>
+      <c r="E4" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G4" t="str">
+        <v>ذكر</v>
+      </c>
+      <c r="H4" t="str">
+        <v>جراحة قلب</v>
+      </c>
+      <c r="I4" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J4" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K4" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="L4" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="M4" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="N4" t="str">
+        <v>عضو أصيل</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v>2026-05-05T17:35:59.270Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve membership application print and email notifications
Update print styles for a professional A4 layout and enhance email notifications with comprehensive HTML content and corrected organization branding.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: fb83f075-83bf-4666-98f0-ea4bec10fd72
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 130d11eb-26a6-4554-9775-abfc54a0a9a0
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/3a6f4480-5f60-41f1-9683-8e05aff8235c/fb83f075-83bf-4666-98f0-ea4bec10fd72/pJCex5R
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/نموذج-الأعضاء-عربي.xlsx
+++ b/docs/form_by_n8n/نموذج-الأعضاء-عربي.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -599,9 +599,59 @@
         <v>2026-05-05T17:35:59.270Z</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ابراهيم</v>
+      </c>
+      <c r="B5" t="str">
+        <v>الصيداوي</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D5" t="str">
+        <v>محمد علي</v>
+      </c>
+      <c r="E5" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G5" t="str">
+        <v>ذكر</v>
+      </c>
+      <c r="H5" t="str">
+        <v>جراحة قلب</v>
+      </c>
+      <c r="I5" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J5" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K5" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="L5" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="M5" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="N5" t="str">
+        <v>عضو أصيل</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v>2026-05-05T17:40:38.322Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Prevent duplicate member entries from being added to the system
Add server-side deduplication logic to prevent multiple entries for the same member.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: fb83f075-83bf-4666-98f0-ea4bec10fd72
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b3e5fda7-da08-42b6-95d4-7a9a1bddd05f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/3a6f4480-5f60-41f1-9683-8e05aff8235c/fb83f075-83bf-4666-98f0-ea4bec10fd72/pJCex5R
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/form_by_n8n/نموذج-الأعضاء-عربي.xlsx
+++ b/docs/form_by_n8n/نموذج-الأعضاء-عربي.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -649,9 +649,109 @@
         <v>2026-05-05T17:40:38.322Z</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ابراهيم</v>
+      </c>
+      <c r="B6" t="str">
+        <v>الصيداوي</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D6" t="str">
+        <v>محمد علي</v>
+      </c>
+      <c r="E6" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G6" t="str">
+        <v>ذكر</v>
+      </c>
+      <c r="H6" t="str">
+        <v>جراحة قلب</v>
+      </c>
+      <c r="I6" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J6" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K6" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="L6" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="M6" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="N6" t="str">
+        <v>عضو أصيل</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v>2026-05-05T17:53:23.829Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ابراهيم</v>
+      </c>
+      <c r="B7" t="str">
+        <v>الصيداوي</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ابراهيم الصيداوي</v>
+      </c>
+      <c r="D7" t="str">
+        <v>محمد علي</v>
+      </c>
+      <c r="E7" t="str">
+        <v>ibrahim sidawi</v>
+      </c>
+      <c r="F7" t="str">
+        <v>1978-04-05</v>
+      </c>
+      <c r="G7" t="str">
+        <v>ذكر</v>
+      </c>
+      <c r="H7" t="str">
+        <v>جراحة قلب</v>
+      </c>
+      <c r="I7" t="str">
+        <v>ibrahimsidawi@gmail.com</v>
+      </c>
+      <c r="J7" t="str">
+        <v>+963933706403</v>
+      </c>
+      <c r="K7" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="L7" t="str">
+        <v>دمشق</v>
+      </c>
+      <c r="M7" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="N7" t="str">
+        <v>عضو أصيل</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v>2026-05-05T17:57:20.590Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>